<commit_message>
투자 대시보드 2026-10-19 18:25
</commit_message>
<xml_diff>
--- a/technicals/exports/2026-10-16.xlsx
+++ b/technicals/exports/2026-10-16.xlsx
@@ -221,7 +221,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 클라우드 기반 인적자본관리 플랫폼과 인사 업무 아웃소싱 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>전 세계에 클라우드 기반 인적자본관리 플랫폼과 인사 업무 아웃소싱을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3">
@@ -300,7 +300,7 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 재산·상해보험을 제공하는 보험 지주회사로, 재산 및 운송보험 상품 등을 취급한다.</ns0:t>
+          <ns0:t>미국에서 재산·상해보험과 운송보험 등을 제공하는 보험 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4">
@@ -458,7 +458,7 @@
       </ns0:c>
       <ns0:c r="F6" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 병원과 의료시설에 기술 기반 의료인력 솔루션 및 인력 공급 서비스를 제공.</ns0:t>
+          <ns0:t>미국 병원·의료시설에 기술 기반 의료인력 솔루션과 인력 공급 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G6">
@@ -537,7 +537,7 @@
       </ns0:c>
       <ns0:c r="F7" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 사격 스포츠 액세서리, 칼 등 야외활동 제품과 용품을 제공하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 사격 스포츠 액세서리·칼 등 야외활동 제품과 용품을 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G7">
@@ -616,7 +616,7 @@
       </ns0:c>
       <ns0:c r="F8" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·이집트·북해에서 천연가스, 원유 및 천연가스액을 탐사·개발·생산하는 독립 에너지 기업.</ns0:t>
+          <ns0:t>미국·이집트·북해에서 천연가스·원유·천연가스액을 탐사·개발·생산하는 독립 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G8">
@@ -695,7 +695,7 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 내 고급 객실 중심 호텔 포트폴리오를 보유한 상장 부동산투자신탁.</ns0:t>
+          <ns0:t>미국 내 고급 객실 중심 호텔을 보유한 상장 부동산투자신탁.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9">
@@ -774,7 +774,7 @@
       </ns0:c>
       <ns0:c r="F10" t="inlineStr">
         <ns0:is>
-          <ns0:t>기업·컨택센터·통신사업자에 음성 통신 인프라·장비, 클라우드 관리 및 음성 AI 솔루션 제공.</ns0:t>
+          <ns0:t>기업·컨택센터·통신사업자에 음성 통신 인프라·장비, 클라우드 관리·음성 AI 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G10">
@@ -932,7 +932,7 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계 의료기관·연구기관 등에 의료용품, 의료기기, 실험실 장비 및 진단 제품을 개발·제조·판매.</ns0:t>
+          <ns0:t>전 세계 의료·연구기관 등에 의료용품·의료기기·실험실 장비·진단 제품을 개발·제조·판매하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12">
@@ -1011,7 +1011,7 @@
       </ns0:c>
       <ns0:c r="F13" t="inlineStr">
         <ns0:is>
-          <ns0:t>다양한 규모의 조직이 장소와 기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
+          <ns0:t>다양한 규모의 조직이 장소·기기에 관계없이 콘텐츠를 관리하는 클라우드 플랫폼 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G13">
@@ -1090,7 +1090,7 @@
       </ns0:c>
       <ns0:c r="F14" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 석유·가스 사업을 운영하며 가스·저탄소 에너지, 석유 생산 및 고객·제품 부문을 영위.</ns0:t>
+          <ns0:t>전 세계에서 가스·저탄소 에너지, 석유 생산, 고객·제품 부문 등 석유·가스 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G14">
@@ -1327,7 +1327,7 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다에서 식당을 운영·라이선스하고, 치즈케이크 등 제과 제품을 생산·공급하는 기업.</ns0:t>
+          <ns0:t>미국·캐나다에서 식당 운영·라이선스 사업과 치즈케이크 등 제과 제품 생산·공급을 하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17">
@@ -1485,7 +1485,7 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>대만과 해외에서 개인·기업 고객에게 이동통신·유선통신 등 통합 통신 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>대만과 해외 개인·기업 고객에게 이동통신·유선통신 등 통합 통신 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19">
@@ -1564,7 +1564,7 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>고급 장기체류 호텔과 프리미엄 브랜드의 선택형 서비스 호텔에 주로 투자하는 상장 부동산투자신탁.</ns0:t>
+          <ns0:t>고급 장기체류 호텔과 프리미엄 브랜드 선택형 서비스 호텔에 주로 투자하는 상장 부동산투자신탁.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20">
@@ -1643,7 +1643,7 @@
       </ns0:c>
       <ns0:c r="F21" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 보험 보장이 부족한 가정과 기업에 프로그램·서비스를 제공하는 관리형 의료 기업.</ns0:t>
+          <ns0:t>미국 내 보험 보장이 부족한 가정·기업에 프로그램과 서비스를 제공하는 관리형 의료 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G21">
@@ -1801,7 +1801,7 @@
       </ns0:c>
       <ns0:c r="F23" t="inlineStr">
         <ns0:is>
-          <ns0:t>캐나다 서부·영국 북해·아프리카 해상에서 원유·천연가스·천연가스액을 탐사·개발·생산·판매하는 기업.</ns0:t>
+          <ns0:t>캐나다 서부·영국 북해·아프리카 해상에서 원유·천연가스·천연가스액을 탐사·개발·생산·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G23">
@@ -1880,7 +1880,7 @@
       </ns0:c>
       <ns0:c r="F24" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소 등을 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
+          <ns0:t>미국에서 직업건강센터와 사업장 내 진료소를 통해 직업건강 및 고용주·소비자 건강 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G24">
@@ -1959,7 +1959,7 @@
       </ns0:c>
       <ns0:c r="F25" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유·역청·천연가스·액화천연가스·천연가스액을 탐사·생산·운송·판매하는 기업.</ns0:t>
+          <ns0:t>원유·역청·천연가스·액화천연가스·천연가스액을 탐사·생산·운송·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G25">
@@ -2038,7 +2038,7 @@
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>원유·천연가스 탐사, 개발, 생산, 운송 등을 포함한 통합 에너지 및 화학 사업을 영위.</ns0:t>
+          <ns0:t>원유·천연가스 탐사·개발·생산·운송 등을 포함한 통합 에너지·화학 사업 영위.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26">
@@ -2196,7 +2196,7 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>한국·미국 등에서 캐주얼 게임과 모바일 앱을 개발·배급하며 소셜 카지노 게임 및 iGaming 사업 운영.</ns0:t>
+          <ns0:t>한국·미국 등에서 캐주얼 게임·모바일 앱을 개발·배급하고 소셜 카지노와 iGaming 사업을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28">
@@ -2433,7 +2433,7 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·트리니다드토바고 등에서 원유·천연가스액·천연가스를 탐사·개발·생산·판매하는 기업.</ns0:t>
+          <ns0:t>미국·트리니다드토바고 등에서 원유·천연가스액·천연가스를 탐사·개발·생산·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31">
@@ -2512,7 +2512,7 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>노르웨이와 해외에서 탐사·생산, 마케팅·미드스트림·가공, 재생에너지 사업을 하는 기업.</ns0:t>
+          <ns0:t>노르웨이와 해외에서 탐사·생산, 마케팅·미드스트림·가공 및 재생에너지 사업을 하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32">
@@ -2591,7 +2591,7 @@
       </ns0:c>
       <ns0:c r="F33" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 구매자와 판매자를 연결하는 Etsy·Depop 온라인 마켓플레이스를 운영하는 기업.</ns0:t>
+          <ns0:t>미국·영국 등에서 구매자와 판매자를 연결하는 Etsy·Depop 온라인 마켓플레이스 운영기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G33">
@@ -2828,7 +2828,7 @@
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>개인·소기업·기업 고객에게 은행·신탁·금융 서비스를 제공하는 은행을 보유한 지주회사.</ns0:t>
+          <ns0:t>개인·소기업·기업에 은행·신탁·금융 서비스를 제공하는 은행을 보유한 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36">
@@ -2907,7 +2907,7 @@
       </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 의료용 의류, 신발 등 생활용품을 소비자에게 직접 판매하는 기업.</ns0:t>
+          <ns0:t>미국과 해외에서 의료용 의류·신발 등 생활용품을 소비자에게 직접 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G37">
@@ -2986,7 +2986,7 @@
       </ns0:c>
       <ns0:c r="F38" t="inlineStr">
         <ns0:is>
-          <ns0:t>증권 중개·매매, 시장조성, 투자 리서치·자문, 소매·상업은행 및 보험 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>증권 중개·매매·시장조성·투자 리서치·자문과 소매·상업은행 및 보험 서비스를 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G38">
@@ -3065,7 +3065,7 @@
       </ns0:c>
       <ns0:c r="F39" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에 고객 경험과 직원 경험을 위한 서비스형 소프트웨어를 제공한다.</ns0:t>
+          <ns0:t>전 세계에 고객·직원 경험을 위한 서비스형 소프트웨어를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G39">
@@ -3144,7 +3144,7 @@
       </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
-          <ns0:t>독자 효소와 기기를 연구·개발·상용화하며 재조합 인간 히알루로니다아제 기반 제품을 보유한 바이오제약사.</ns0:t>
+          <ns0:t>독자 효소·기기를 연구·개발·상용화하며 재조합 인간 히알루로니다아제 기반 제품을 보유한 바이오제약사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G40">
@@ -3223,7 +3223,7 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험을 제공하며 보험·마켓플레이스 부문을 운영.</ns0:t>
+          <ns0:t>미국·캐나다·영국에서 수집용·자동차 애호가용 차량 보험과 마켓플레이스 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41">
@@ -3302,7 +3302,7 @@
       </ns0:c>
       <ns0:c r="F42" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 오토바이·자동차·동력 제품을 개발·제조·유통하고 금융 서비스를 제공하는 기업.</ns0:t>
+          <ns0:t>세계 각지에서 오토바이·자동차·동력 제품을 개발·제조·유통하고 금융 서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G42">
@@ -3460,7 +3460,7 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공하는 기업.</ns0:t>
+          <ns0:t>기술 기반 고객 경험 솔루션과 고객서비스·기술지원·백오피스 아웃소싱을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44">
@@ -3539,7 +3539,7 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 소비재 브랜드 등의 디지털 판촉을 제휴 매체 네트워크를 통해 소비자에게 제공.</ns0:t>
+          <ns0:t>미국 소비재 브랜드 등의 디지털 판촉을 제휴 매체 네트워크로 소비자에게 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45">
@@ -3618,7 +3618,7 @@
       </ns0:c>
       <ns0:c r="F46" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션을 제공하는 기업.</ns0:t>
+          <ns0:t>미국·영국 등에서 핀테크 및 통신 솔루션 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G46">
@@ -3697,7 +3697,7 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>식품·음료·건강 및 바이오과학·향료와 관련 제품을 제조·판매하는 글로벌 기업.</ns0:t>
+          <ns0:t>식품·음료·건강·바이오과학·향료 관련 제품을 제조·판매하는 글로벌 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47">
@@ -3776,7 +3776,7 @@
       </ns0:c>
       <ns0:c r="F48" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 장난감, 소비재·전자제품, 아동용 가구, 의상, 스포츠용품, 가정용 가구 등을 제작·판매.</ns0:t>
+          <ns0:t>전 세계에서 장난감, 소비재·전자제품, 아동·가정용 가구, 의상, 스포츠용품을 제작·판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G48">
@@ -3855,7 +3855,7 @@
       </ns0:c>
       <ns0:c r="F49" t="inlineStr">
         <ns0:is>
-          <ns0:t>주요 영업활동 없이 방위·항공우주 분야 기업과의 합병, 주식 교환, 인수 등 기업결합을 추진한다.</ns0:t>
+          <ns0:t>주요 영업활동 없이 방위·항공우주 기업과 합병·주식 교환·인수 등 기업결합을 추진한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G49">
@@ -4010,7 +4010,7 @@
       </ns0:c>
       <ns0:c r="F51" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 석유·가스 에너지 사업을 발굴·개발하며 오클라호마 캐니 셰일 유전을 개발하는 기업.</ns0:t>
+          <ns0:t>미국에서 석유·가스 사업을 발굴·개발하고 오클라호마 캐니 셰일 유전을 개발하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G51">
@@ -4168,7 +4168,7 @@
       </ns0:c>
       <ns0:c r="F53" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 석유·천연가스 자산의 광물권과 로열티 권익을 보유·취득하는 기업.</ns0:t>
+          <ns0:t>미국 석유·천연가스 자산의 광물권과 로열티 권익을 보유·취득.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G53">
@@ -4247,7 +4247,7 @@
       </ns0:c>
       <ns0:c r="F54" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 거래 처리 및 결제 관련 제품·서비스를 소비자, 가맹점, 금융기관 등에 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 소비자·가맹점·금융기관 등에 거래 처리와 결제 제품·서비스를 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G54">
@@ -4326,7 +4326,7 @@
       </ns0:c>
       <ns0:c r="F55" t="inlineStr">
         <ns0:is>
-          <ns0:t>공급망·재고·옴니채널 운영과 창고 관리를 위한 소프트웨어를 개발·판매·구축·유지보수.</ns0:t>
+          <ns0:t>공급망·재고·옴니채널 운영·창고 관리 소프트웨어를 개발·판매·구축·유지보수하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G55">
@@ -4405,7 +4405,7 @@
       </ns0:c>
       <ns0:c r="F56" t="inlineStr">
         <ns0:is>
-          <ns0:t>의약품 유통, 종양·전문진료, 처방 기술, 의료·외과용품 관련 의료 서비스를 제공.</ns0:t>
+          <ns0:t>의약품 유통·종양 및 전문진료·처방 기술·의료 및 외과용품 관련 의료 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G56">
@@ -4484,7 +4484,7 @@
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 신생아·모체태아·소아 세부전문 진료와 미숙아·합병증 신생아 치료를 제공하는 기업.</ns0:t>
+          <ns0:t>미국에서 신생아·모체태아·소아 전문 진료와 미숙아·합병증 신생아 치료를 제공하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57">
@@ -4563,7 +4563,7 @@
       </ns0:c>
       <ns0:c r="F58" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 보험, 연금, 임직원 복리후생 및 자산관리 서비스를 제공하는 금융서비스 기업.</ns0:t>
+          <ns0:t>전 세계에서 보험·연금·임직원 복리후생·자산관리 서비스를 제공하는 금융서비스 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G58">
@@ -4721,7 +4721,7 @@
       </ns0:c>
       <ns0:c r="F60" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 식음료 판매, 컨설팅, 전자폐기물 자재 판매 등 공급망 사업을 운영한다.</ns0:t>
+          <ns0:t>미국에서 식음료 판매, 컨설팅, 전자폐기물 자재 판매 등 공급망 사업을 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G60">
@@ -4800,7 +4800,7 @@
       </ns0:c>
       <ns0:c r="F61" t="inlineStr">
         <ns0:is>
-          <ns0:t>전문 간호·생활지원·독립생활 시설, 재택돌봄·호스피스 기관 및 병원 서비스를 운영하는 기업.</ns0:t>
+          <ns0:t>전문 간호·생활지원·독립생활 시설과 재택돌봄·호스피스 기관 및 병원 서비스를 운영하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G61">
@@ -4958,7 +4958,7 @@
       </ns0:c>
       <ns0:c r="F63" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 온라인·전화·매장 및 제휴 채널을 통해 개인대출과 신용카드를 제공.</ns0:t>
+          <ns0:t>미국에서 온라인·전화·매장 및 제휴 채널을 통해 개인대출과 신용카드 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G63">
@@ -5116,7 +5116,7 @@
       </ns0:c>
       <ns0:c r="F65" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국 중소·중견기업에 채용 등 고용 전 과정을 관리하는 클라우드 인적자본관리 소프트웨어를 제공.</ns0:t>
+          <ns0:t>미국 중소·중견기업에 채용 등 고용 전 과정을 관리하는 클라우드 인적자본관리 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G65">
@@ -5195,7 +5195,7 @@
       </ns0:c>
       <ns0:c r="F66" t="inlineStr">
         <ns0:is>
-          <ns0:t>선불카드, 환자 비용 부담 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
+          <ns0:t>선불카드, 환자 비용 지원, 디지털뱅킹, 생명과학 소프트웨어 및 통합 결제처리를 제공하는 회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G66">
@@ -5274,7 +5274,7 @@
       </ns0:c>
       <ns0:c r="F67" t="inlineStr">
         <ns0:is>
-          <ns0:t>브라질과 해외에서 석유·가스를 탐사·생산·판매하며 정유·운송·판매 사업을 운영한다.</ns0:t>
+          <ns0:t>브라질과 해외에서 석유·가스 탐사·생산·판매 및 정유·운송 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G67">
@@ -5353,7 +5353,7 @@
       </ns0:c>
       <ns0:c r="F68" t="inlineStr">
         <ns0:is>
-          <ns0:t>브라질과 해외에서 석유·가스를 탐사·생산·판매하며 정유·운송·판매 사업을 운영한다.</ns0:t>
+          <ns0:t>브라질과 해외에서 석유·가스 탐사·생산·판매 및 정유·운송 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G68">
@@ -5432,7 +5432,7 @@
       </ns0:c>
       <ns0:c r="F69" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 급여·세무·인사 관리 등을 지원하는 클라우드 인적자본관리·재무·IT 소프트웨어를 제공.</ns0:t>
+          <ns0:t>미국에서 급여·세무·인사 관리를 지원하는 클라우드 인적자본관리·재무·IT 소프트웨어 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G69">
@@ -5590,7 +5590,7 @@
       </ns0:c>
       <ns0:c r="F71" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국의 도심·리조트형 라이프스타일 호텔을 보유한 상장 부동산투자신탁.</ns0:t>
+          <ns0:t>미국 도심·리조트형 라이프스타일 호텔을 보유한 상장 부동산투자신탁.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G71">
@@ -5748,7 +5748,7 @@
       </ns0:c>
       <ns0:c r="F73" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 교육 교재·평가·자격인증·온라인 학습·영어 학습 등 교육 서비스를 제공.</ns0:t>
+          <ns0:t>세계 각지에서 교육 교재·평가·자격인증·온라인 학습·영어 학습 등 교육 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G73">
@@ -5827,7 +5827,7 @@
       </ns0:c>
       <ns0:c r="F74" t="inlineStr">
         <ns0:is>
-          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산.</ns0:t>
+          <ns0:t>텍사스·뉴멕시코에서 석유·천연가스·천연가스액 자산을 인수·탐사·개발·생산한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G74">
@@ -5906,7 +5906,7 @@
       </ns0:c>
       <ns0:c r="F75" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계에서 생명·건강 및 자산집약형 재보험을 제공하며 장애·장기요양 관련 보장도 취급.</ns0:t>
+          <ns0:t>전 세계에서 생명·건강·자산집약형 재보험을 제공하고 장애·장기요양 관련 보장도 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G75">
@@ -5985,7 +5985,7 @@
       </ns0:c>
       <ns0:c r="F76" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 재산·상해·특종 보험과 재보험을 제공하며 재산 재해 초과손해 재보험을 취급.</ns0:t>
+          <ns0:t>미국과 해외에서 재산·상해·특종 보험 및 재보험을 제공하고 재산 재해 초과손해 재보험 취급.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G76">
@@ -6143,7 +6143,7 @@
       </ns0:c>
       <ns0:c r="F78" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 건강한 음식과 음료를 제공하는 패스트푸드 식당을 운영하며 온라인·모바일 주문을 지원.</ns0:t>
+          <ns0:t>미국에서 건강한 음식·음료를 제공하는 패스트푸드 식당을 운영하고 온라인·모바일 주문 지원.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G78">
@@ -6222,7 +6222,7 @@
       </ns0:c>
       <ns0:c r="F79" t="inlineStr">
         <ns0:is>
-          <ns0:t>세계 각지에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
+          <ns0:t>전 세계에서 통합 가스, 자원 개발·생산, 마케팅, 화학·제품, 재생에너지 사업을 운영한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G79">
@@ -6301,7 +6301,7 @@
       </ns0:c>
       <ns0:c r="F80" t="inlineStr">
         <ns0:is>
-          <ns0:t>입지가 좋은 호텔·리조트 부동산을 인수·적극 운영·매각하는 숙박 부동산투자신탁.</ns0:t>
+          <ns0:t>입지가 좋은 호텔·리조트 부동산을 인수·운영·매각하는 숙박 부동산투자신탁.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G80">
@@ -6380,7 +6380,7 @@
       </ns0:c>
       <ns0:c r="F81" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다·영국·아일랜드에서 다이아몬드 주얼리 소매점을 운영.</ns0:t>
+          <ns0:t>미국·캐나다·영국·아일랜드에서 다이아몬드 주얼리 소매점을 운영하는 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G81">
@@ -6459,7 +6459,7 @@
       </ns0:c>
       <ns0:c r="F82" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국에서 해안 지역 주택·콘도·상업용 주거시설 등의 손해보험과 재보험·보험대리 서비스를 제공.</ns0:t>
+          <ns0:t>미국 해안 지역 주택·콘도·상업용 주거시설의 손해보험과 재보험·보험대리 서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G82">
@@ -6538,7 +6538,7 @@
       </ns0:c>
       <ns0:c r="F83" t="inlineStr">
         <ns0:is>
-          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청, 연료, 나프타, 윤활유, 액화석유가스 등을 공급한다.</ns0:t>
+          <ns0:t>남아공 등에서 화학·에너지 사업을 운영하며 역청·연료·나프타·윤활유·액화석유가스를 공급한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G83">
@@ -6617,7 +6617,7 @@
       </ns0:c>
       <ns0:c r="F84" t="inlineStr">
         <ns0:is>
-          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 영위하는 종합 에너지 기업.</ns0:t>
+          <ns0:t>캐나다·미국 등에서 오일샌드, 석유 탐사·생산, 정유·판매 사업을 운영하는 종합 에너지 기업.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G84">
@@ -6930,7 +6930,7 @@
       </ns0:c>
       <ns0:c r="F88" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 소매·도매·구독 사업으로 의류·신발·액세서리 등 라이프스타일 상품과 서비스 제공.</ns0:t>
+          <ns0:t>미국과 해외에서 소매·도매·구독 사업을 통해 의류·신발·액세서리 등 라이프스타일 상품·서비스 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G88">
@@ -7088,7 +7088,7 @@
       </ns0:c>
       <ns0:c r="F90" t="inlineStr">
         <ns0:is>
-          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공.</ns0:t>
+          <ns0:t>결제 승인·청산·정산 네트워크 VisaNet을 운영하고 신용·직불·선불카드 상품을 제공한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G90">
@@ -7167,7 +7167,7 @@
       </ns0:c>
       <ns0:c r="F91" t="inlineStr">
         <ns0:is>
-          <ns0:t>버지니아 내 상업·개인 금융 서비스를 제공하는 은행의 지주회사로 은행 및 신탁·상속재산 서비스 운영.</ns0:t>
+          <ns0:t>버지니아에서 상업·개인 금융과 신탁·상속재산 서비스를 운영하는 은행 지주회사.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G91">
@@ -7246,7 +7246,7 @@
       </ns0:c>
       <ns0:c r="F92" t="inlineStr">
         <ns0:is>
-          <ns0:t>전 세계 생명과학 산업에 클라우드 소프트웨어를 제공하며 제약·바이오 기업용 CRM 제품군 등을 제공.</ns0:t>
+          <ns0:t>전 세계 생명과학 산업에 클라우드 소프트웨어와 제약·바이오 기업용 CRM 제품군 등을 제공.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G92">
@@ -7325,7 +7325,7 @@
       </ns0:c>
       <ns0:c r="F93" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 도매·소비자 직접판매 사업을 운영하며 캐시미어 스웨터·실크 블라우스 등 여성복을 판매한다.</ns0:t>
+          <ns0:t>미국과 해외에서 도매·소비자 직접판매로 캐시미어 스웨터·실크 블라우스 등 여성복을 판매한다.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G93">
@@ -7641,7 +7641,7 @@
       </ns0:c>
       <ns0:c r="F97" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외에서 온·오프라인으로 조리·식사·접객용품과 가구 등 가정용 제품을 판매.</ns0:t>
+          <ns0:t>미국과 해외 온·오프라인에서 조리·식사·접객용품과 가구 등 가정용 제품 판매.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G97">
@@ -7799,7 +7799,7 @@
       </ns0:c>
       <ns0:c r="F99" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국·캐나다 등에서 원유·천연가스를 탐사·생산하며 에너지·화학·특수제품 사업을 운영한다.</ns0:t>
+          <ns0:t>미국·캐나다 등에서 원유·천연가스를 탐사·생산하며 에너지·화학·특수제품 사업 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G99">
@@ -7878,7 +7878,7 @@
       </ns0:c>
       <ns0:c r="F100" t="inlineStr">
         <ns0:is>
-          <ns0:t>미국과 해외 기업에 소비자 인텔리전스와 마케팅 자동화 소프트웨어를 제공하는 옴니채널 데이터 기반 플랫폼 운영.</ns0:t>
+          <ns0:t>미국과 해외 기업에 소비자 인텔리전스·마케팅 자동화 소프트웨어를 제공하는 옴니채널 데이터 기반 플랫폼 운영.</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G100">

</xml_diff>